<commit_message>
temporary including 2CC now removing it
</commit_message>
<xml_diff>
--- a/Constrained_BO/results/final_charging_opt_results/RW10/comparison_table.xlsx
+++ b/Constrained_BO/results/final_charging_opt_results/RW10/comparison_table.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -528,7 +528,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>
@@ -540,34 +540,44 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CC 1C</t>
+          <t>CCCV 1C</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>18.97</v>
+        <v>25.17</v>
       </c>
       <c r="D3" t="n">
-        <v>34.22</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="E3" t="n">
+        <v>20.53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>79.47</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="I3" t="n">
+        <v>45.43</v>
+      </c>
       <c r="J3" t="n">
-        <v>26.5</v>
+        <v>24.11</v>
       </c>
       <c r="K3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>infeasible (energy target not met)</t>
+          <t>feasible</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>
@@ -579,34 +589,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CC 2C</t>
+          <t>CCCV 2C</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5.6</v>
+        <v>28.02</v>
       </c>
       <c r="D4" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+        <v>40</v>
+      </c>
+      <c r="E4" t="n">
+        <v>20.82</v>
+      </c>
+      <c r="F4" t="n">
+        <v>79.18000000000001</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.82</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-3.88</v>
+      </c>
+      <c r="I4" t="n">
+        <v>39.25</v>
+      </c>
       <c r="J4" t="n">
-        <v>29.4</v>
+        <v>24.3</v>
       </c>
       <c r="K4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>infeasible (energy target not met)</t>
+          <t>feasible</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>
@@ -655,7 +675,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>
@@ -704,7 +724,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>
@@ -753,7 +773,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>CC ½C</t>
+          <t>CCCV ½C</t>
         </is>
       </c>
     </row>

</xml_diff>